<commit_message>
Add links as sources, and modify the location of the edit system prompt.
</commit_message>
<xml_diff>
--- a/Docs & Links/Docs & Links - Chatbot P&R Hub.xlsx
+++ b/Docs & Links/Docs & Links - Chatbot P&R Hub.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="326" uniqueCount="191">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="326" uniqueCount="193">
   <si>
     <t>NAME DOCUMENT</t>
   </si>
@@ -64,6 +64,9 @@
     </r>
   </si>
   <si>
+    <t>Portfolio Narrative_2024.pdf</t>
+  </si>
+  <si>
     <t>https://cgspace.cgiar.org/items/04bd63a9-1b58-4eb5-84f2-b54c8bde226e</t>
   </si>
   <si>
@@ -79,6 +82,9 @@
       </rPr>
       <t>https://storage.googleapis.com/cgiarorg/2025/06/CGIAR-Technical-Reporting-Arrangement-2025-30.pdf</t>
     </r>
+  </si>
+  <si>
+    <t>Type3_2024Report.pdf</t>
   </si>
   <si>
     <r>
@@ -1694,10 +1700,10 @@
     </row>
     <row r="5">
       <c r="A5" s="4" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C5" s="6" t="s">
         <v>4</v>
@@ -1709,10 +1715,10 @@
     </row>
     <row r="6">
       <c r="A6" s="4" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C6" s="6" t="s">
         <v>4</v>
@@ -1724,10 +1730,10 @@
     </row>
     <row r="7">
       <c r="A7" s="4" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="C7" s="6" t="s">
         <v>4</v>
@@ -1739,10 +1745,10 @@
     </row>
     <row r="8">
       <c r="A8" s="4" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C8" s="6" t="s">
         <v>4</v>
@@ -1754,10 +1760,10 @@
     </row>
     <row r="9">
       <c r="A9" s="4" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C9" s="6" t="s">
         <v>4</v>
@@ -1769,10 +1775,10 @@
     </row>
     <row r="10">
       <c r="A10" s="4" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C10" s="6" t="s">
         <v>4</v>
@@ -1784,10 +1790,10 @@
     </row>
     <row r="11">
       <c r="A11" s="4" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C11" s="6" t="s">
         <v>4</v>
@@ -1797,10 +1803,10 @@
     </row>
     <row r="12">
       <c r="A12" s="4" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C12" s="6" t="s">
         <v>4</v>
@@ -1810,10 +1816,10 @@
     </row>
     <row r="13">
       <c r="A13" s="4" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C13" s="6" t="s">
         <v>4</v>
@@ -1825,16 +1831,16 @@
     </row>
     <row r="14">
       <c r="A14" s="4" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B14" s="9" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D14" s="8" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="E14" s="6" t="s">
         <v>4</v>
@@ -1842,10 +1848,10 @@
     </row>
     <row r="15">
       <c r="A15" s="4" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C15" s="6" t="s">
         <v>4</v>
@@ -1857,16 +1863,16 @@
     </row>
     <row r="16">
       <c r="A16" s="4" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D16" s="8" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="E16" s="6" t="s">
         <v>4</v>
@@ -1874,10 +1880,10 @@
     </row>
     <row r="17">
       <c r="A17" s="4" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C17" s="6" t="s">
         <v>4</v>
@@ -1889,10 +1895,10 @@
     </row>
     <row r="18">
       <c r="A18" s="4" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C18" s="6" t="s">
         <v>4</v>
@@ -1904,16 +1910,16 @@
     </row>
     <row r="19">
       <c r="A19" s="4" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B19" s="9" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D19" s="8" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="E19" s="6" t="s">
         <v>4</v>
@@ -1921,16 +1927,16 @@
     </row>
     <row r="20">
       <c r="A20" s="4" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B20" s="9" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D20" s="8" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="E20" s="6" t="s">
         <v>4</v>
@@ -1938,16 +1944,16 @@
     </row>
     <row r="21">
       <c r="A21" s="4" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="B21" s="9" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D21" s="8" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="E21" s="6" t="s">
         <v>4</v>
@@ -1955,10 +1961,10 @@
     </row>
     <row r="22">
       <c r="A22" s="4" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="B22" s="8" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="C22" s="6" t="s">
         <v>4</v>
@@ -1970,16 +1976,16 @@
     </row>
     <row r="23">
       <c r="A23" s="4" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="B23" s="9" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C23" s="6" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D23" s="8" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="E23" s="6" t="s">
         <v>4</v>
@@ -1987,10 +1993,10 @@
     </row>
     <row r="24">
       <c r="A24" s="4" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="B24" s="8" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="C24" s="6" t="s">
         <v>4</v>
@@ -2002,16 +2008,16 @@
     </row>
     <row r="25">
       <c r="A25" s="4" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B25" s="9" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C25" s="6" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D25" s="8" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="E25" s="6" t="s">
         <v>4</v>
@@ -2019,16 +2025,16 @@
     </row>
     <row r="26">
       <c r="A26" s="4" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B26" s="9" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C26" s="6" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D26" s="8" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="E26" s="6" t="s">
         <v>4</v>
@@ -2036,10 +2042,10 @@
     </row>
     <row r="27">
       <c r="A27" s="4" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B27" s="8" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C27" s="6" t="s">
         <v>4</v>
@@ -2051,10 +2057,10 @@
     </row>
     <row r="28">
       <c r="A28" s="4" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B28" s="8" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C28" s="6" t="s">
         <v>4</v>
@@ -2066,16 +2072,16 @@
     </row>
     <row r="29">
       <c r="A29" s="4" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B29" s="9" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C29" s="6" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D29" s="8" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="E29" s="6" t="s">
         <v>4</v>
@@ -2083,10 +2089,10 @@
     </row>
     <row r="30">
       <c r="A30" s="4" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B30" s="8" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="C30" s="6" t="s">
         <v>4</v>
@@ -2098,10 +2104,10 @@
     </row>
     <row r="31">
       <c r="A31" s="4" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B31" s="8" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C31" s="6" t="s">
         <v>4</v>
@@ -2113,16 +2119,16 @@
     </row>
     <row r="32">
       <c r="A32" s="4" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B32" s="9" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C32" s="6" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D32" s="8" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="E32" s="6" t="s">
         <v>4</v>
@@ -2130,10 +2136,10 @@
     </row>
     <row r="33">
       <c r="A33" s="4" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B33" s="5" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="C33" s="6" t="s">
         <v>4</v>
@@ -2143,10 +2149,10 @@
     </row>
     <row r="34">
       <c r="A34" s="4" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="C34" s="6" t="s">
         <v>4</v>
@@ -2156,10 +2162,10 @@
     </row>
     <row r="35">
       <c r="A35" s="4" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B35" s="5" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C35" s="6" t="s">
         <v>4</v>
@@ -2169,10 +2175,10 @@
     </row>
     <row r="36">
       <c r="A36" s="4" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B36" s="5" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="C36" s="6" t="s">
         <v>4</v>
@@ -2182,10 +2188,10 @@
     </row>
     <row r="37">
       <c r="A37" s="4" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B37" s="5" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C37" s="6" t="s">
         <v>4</v>
@@ -2195,10 +2201,10 @@
     </row>
     <row r="38">
       <c r="A38" s="4" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B38" s="5" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="C38" s="6" t="s">
         <v>4</v>
@@ -2208,10 +2214,10 @@
     </row>
     <row r="39">
       <c r="A39" s="4" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B39" s="5" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="C39" s="6" t="s">
         <v>4</v>
@@ -2221,10 +2227,10 @@
     </row>
     <row r="40">
       <c r="A40" s="4" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B40" s="5" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="C40" s="6" t="s">
         <v>4</v>
@@ -2234,10 +2240,10 @@
     </row>
     <row r="41">
       <c r="A41" s="4" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B41" s="5" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C41" s="6" t="s">
         <v>4</v>
@@ -2247,10 +2253,10 @@
     </row>
     <row r="42">
       <c r="A42" s="4" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B42" s="5" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="C42" s="6" t="s">
         <v>4</v>
@@ -2260,10 +2266,10 @@
     </row>
     <row r="43">
       <c r="A43" s="4" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B43" s="5" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="C43" s="6" t="s">
         <v>4</v>
@@ -2273,10 +2279,10 @@
     </row>
     <row r="44">
       <c r="A44" s="4" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="B44" s="5" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="C44" s="6" t="s">
         <v>4</v>
@@ -2286,10 +2292,10 @@
     </row>
     <row r="45">
       <c r="A45" s="4" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="B45" s="5" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C45" s="6" t="s">
         <v>4</v>
@@ -2299,10 +2305,10 @@
     </row>
     <row r="46">
       <c r="A46" s="4" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="B46" s="5" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C46" s="6" t="s">
         <v>4</v>
@@ -2312,10 +2318,10 @@
     </row>
     <row r="47">
       <c r="A47" s="4" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="B47" s="5" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="C47" s="6" t="s">
         <v>4</v>
@@ -2325,10 +2331,10 @@
     </row>
     <row r="48">
       <c r="A48" s="4" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B48" s="5" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="C48" s="6" t="s">
         <v>4</v>
@@ -2338,10 +2344,10 @@
     </row>
     <row r="49">
       <c r="A49" s="4" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="B49" s="5" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="C49" s="6" t="s">
         <v>4</v>
@@ -2351,10 +2357,10 @@
     </row>
     <row r="50">
       <c r="A50" s="4" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B50" s="5" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="C50" s="6" t="s">
         <v>4</v>
@@ -2364,10 +2370,10 @@
     </row>
     <row r="51">
       <c r="A51" s="4" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B51" s="5" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="C51" s="6" t="s">
         <v>4</v>
@@ -2377,10 +2383,10 @@
     </row>
     <row r="52">
       <c r="A52" s="4" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="B52" s="5" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="C52" s="6" t="s">
         <v>4</v>
@@ -2390,10 +2396,10 @@
     </row>
     <row r="53">
       <c r="A53" s="4" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B53" s="5" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="C53" s="6" t="s">
         <v>4</v>
@@ -2403,10 +2409,10 @@
     </row>
     <row r="54">
       <c r="A54" s="4" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="B54" s="5" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="C54" s="6" t="s">
         <v>4</v>
@@ -2416,10 +2422,10 @@
     </row>
     <row r="55">
       <c r="A55" s="4" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="B55" s="5" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="C55" s="6" t="s">
         <v>4</v>
@@ -2429,10 +2435,10 @@
     </row>
     <row r="56">
       <c r="A56" s="4" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="B56" s="5" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="C56" s="6" t="s">
         <v>4</v>
@@ -2442,10 +2448,10 @@
     </row>
     <row r="57">
       <c r="A57" s="4" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B57" s="5" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="C57" s="6" t="s">
         <v>4</v>
@@ -2455,10 +2461,10 @@
     </row>
     <row r="58">
       <c r="A58" s="4" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="B58" s="5" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="C58" s="6" t="s">
         <v>4</v>
@@ -2468,10 +2474,10 @@
     </row>
     <row r="59">
       <c r="A59" s="4" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B59" s="5" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="C59" s="6" t="s">
         <v>4</v>
@@ -2481,10 +2487,10 @@
     </row>
     <row r="60">
       <c r="A60" s="4" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="B60" s="5" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C60" s="6" t="s">
         <v>4</v>
@@ -2494,10 +2500,10 @@
     </row>
     <row r="61">
       <c r="A61" s="4" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="B61" s="5" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="C61" s="6" t="s">
         <v>4</v>
@@ -2507,10 +2513,10 @@
     </row>
     <row r="62">
       <c r="A62" s="4" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="B62" s="5" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="C62" s="6" t="s">
         <v>4</v>
@@ -2520,10 +2526,10 @@
     </row>
     <row r="63">
       <c r="A63" s="4" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="B63" s="5" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="C63" s="6" t="s">
         <v>4</v>
@@ -2533,10 +2539,10 @@
     </row>
     <row r="64">
       <c r="A64" s="4" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B64" s="5" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="C64" s="6" t="s">
         <v>4</v>
@@ -2546,10 +2552,10 @@
     </row>
     <row r="65">
       <c r="A65" s="4" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="B65" s="5" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C65" s="6" t="s">
         <v>4</v>
@@ -2559,10 +2565,10 @@
     </row>
     <row r="66">
       <c r="A66" s="4" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B66" s="5" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="C66" s="6" t="s">
         <v>4</v>
@@ -2572,10 +2578,10 @@
     </row>
     <row r="67">
       <c r="A67" s="4" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="B67" s="5" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="C67" s="6" t="s">
         <v>4</v>
@@ -2585,10 +2591,10 @@
     </row>
     <row r="68">
       <c r="A68" s="4" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="B68" s="5" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="C68" s="6" t="s">
         <v>4</v>
@@ -2598,10 +2604,10 @@
     </row>
     <row r="69">
       <c r="A69" s="4" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B69" s="5" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="C69" s="6" t="s">
         <v>4</v>
@@ -2611,10 +2617,10 @@
     </row>
     <row r="70">
       <c r="A70" s="4" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="B70" s="5" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="C70" s="6" t="s">
         <v>4</v>
@@ -2624,10 +2630,10 @@
     </row>
     <row r="71">
       <c r="A71" s="4" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B71" s="5" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="C71" s="6" t="s">
         <v>4</v>
@@ -2637,10 +2643,10 @@
     </row>
     <row r="72">
       <c r="A72" s="4" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="B72" s="5" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="C72" s="6" t="s">
         <v>4</v>
@@ -2650,10 +2656,10 @@
     </row>
     <row r="73">
       <c r="A73" s="4" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="B73" s="5" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="C73" s="6" t="s">
         <v>4</v>
@@ -2663,10 +2669,10 @@
     </row>
     <row r="74">
       <c r="A74" s="4" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="B74" s="5" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="C74" s="6" t="s">
         <v>4</v>
@@ -2676,10 +2682,10 @@
     </row>
     <row r="75">
       <c r="A75" s="4" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="B75" s="5" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="C75" s="6" t="s">
         <v>4</v>
@@ -2689,10 +2695,10 @@
     </row>
     <row r="76">
       <c r="A76" s="4" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="B76" s="5" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="C76" s="6" t="s">
         <v>4</v>
@@ -2702,10 +2708,10 @@
     </row>
     <row r="77">
       <c r="A77" s="4" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="B77" s="5" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="C77" s="6" t="s">
         <v>4</v>
@@ -2715,10 +2721,10 @@
     </row>
     <row r="78">
       <c r="A78" s="4" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="B78" s="5" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="C78" s="6" t="s">
         <v>4</v>
@@ -2728,10 +2734,10 @@
     </row>
     <row r="79">
       <c r="A79" s="4" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="B79" s="5" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="C79" s="6" t="s">
         <v>4</v>
@@ -2741,10 +2747,10 @@
     </row>
     <row r="80">
       <c r="A80" s="4" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="B80" s="5" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="C80" s="6" t="s">
         <v>4</v>
@@ -2754,10 +2760,10 @@
     </row>
     <row r="81">
       <c r="A81" s="4" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="B81" s="5" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="C81" s="6" t="s">
         <v>4</v>
@@ -2767,10 +2773,10 @@
     </row>
     <row r="82">
       <c r="A82" s="4" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="B82" s="5" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="C82" s="6" t="s">
         <v>4</v>
@@ -2780,10 +2786,10 @@
     </row>
     <row r="83">
       <c r="A83" s="4" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="B83" s="5" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="C83" s="6" t="s">
         <v>4</v>
@@ -2793,10 +2799,10 @@
     </row>
     <row r="84">
       <c r="A84" s="4" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="B84" s="5" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="C84" s="6" t="s">
         <v>4</v>
@@ -2806,10 +2812,10 @@
     </row>
     <row r="85">
       <c r="A85" s="4" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="B85" s="5" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="C85" s="6" t="s">
         <v>4</v>
@@ -2819,10 +2825,10 @@
     </row>
     <row r="86">
       <c r="A86" s="4" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="B86" s="5" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="C86" s="6" t="s">
         <v>4</v>
@@ -2832,10 +2838,10 @@
     </row>
     <row r="87">
       <c r="A87" s="4" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="B87" s="5" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="C87" s="6" t="s">
         <v>4</v>
@@ -2845,10 +2851,10 @@
     </row>
     <row r="88">
       <c r="A88" s="4" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="B88" s="5" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="C88" s="6" t="s">
         <v>4</v>
@@ -2858,10 +2864,10 @@
     </row>
     <row r="89">
       <c r="A89" s="4" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="B89" s="5" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="C89" s="6" t="s">
         <v>4</v>
@@ -2871,10 +2877,10 @@
     </row>
     <row r="90">
       <c r="A90" s="4" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="B90" s="5" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="C90" s="6" t="s">
         <v>4</v>
@@ -2884,10 +2890,10 @@
     </row>
     <row r="91">
       <c r="A91" s="4" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="B91" s="5" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="C91" s="6" t="s">
         <v>4</v>
@@ -2897,10 +2903,10 @@
     </row>
     <row r="92">
       <c r="A92" s="4" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="B92" s="5" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="C92" s="6" t="s">
         <v>4</v>
@@ -2910,10 +2916,10 @@
     </row>
     <row r="93">
       <c r="A93" s="4" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="B93" s="5" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="C93" s="6" t="s">
         <v>4</v>
@@ -2923,10 +2929,10 @@
     </row>
     <row r="94">
       <c r="A94" s="4" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="B94" s="5" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="C94" s="6" t="s">
         <v>4</v>
@@ -2936,10 +2942,10 @@
     </row>
     <row r="95">
       <c r="A95" s="4" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="B95" s="9" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="C95" s="6" t="s">
         <v>4</v>
@@ -2949,10 +2955,10 @@
     </row>
     <row r="96">
       <c r="A96" s="4" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="B96" s="5" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="C96" s="6" t="s">
         <v>4</v>

</xml_diff>